<commit_message>
Date and time mention on web
</commit_message>
<xml_diff>
--- a/terraform_modules_service_tracker V1.1.xlsx
+++ b/terraform_modules_service_tracker V1.1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ingrammicro-my.sharepoint.com/personal/jeetendra_wadhwani_ingrammicro_com/Documents/Desktop/terraform-aws-delivery/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="29" documentId="13_ncr:1_{F7EB1B05-2536-42C3-822D-4580F810F1EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{47E45865-DF43-4BC7-BCBE-D5981F8A2349}"/>
+  <xr:revisionPtr revIDLastSave="35" documentId="13_ncr:1_{F7EB1B05-2536-42C3-822D-4580F810F1EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E5BB8156-C9AF-40BD-B896-2C0B5F47F45E}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="268" uniqueCount="137">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="268" uniqueCount="138">
   <si>
     <t>Category</t>
   </si>
@@ -434,6 +434,9 @@
   </si>
   <si>
     <t>Check open SGs, public S3, unencrypted volumes</t>
+  </si>
+  <si>
+    <t>yes</t>
   </si>
 </sst>
 </file>
@@ -1057,10 +1060,10 @@
       <c r="H9" s="3"/>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A10" s="4" t="s">
+      <c r="A10" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="B10" s="5" t="s">
         <v>31</v>
       </c>
       <c r="C10" s="3" t="s">
@@ -1070,21 +1073,21 @@
         <v>33</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>34</v>
+        <v>12</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>34</v>
+        <v>12</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>35</v>
+        <v>13</v>
       </c>
       <c r="H10" s="3"/>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A11" s="4" t="s">
+      <c r="A11" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="B11" s="5" t="s">
         <v>36</v>
       </c>
       <c r="C11" s="3" t="s">
@@ -1094,13 +1097,13 @@
         <v>38</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>34</v>
+        <v>12</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>34</v>
+        <v>12</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>35</v>
+        <v>13</v>
       </c>
       <c r="H11" s="3"/>
     </row>
@@ -1419,10 +1422,10 @@
       <c r="H24" s="3"/>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A25" s="3" t="s">
+      <c r="A25" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="B25" s="3" t="s">
+      <c r="B25" s="5" t="s">
         <v>85</v>
       </c>
       <c r="C25" s="3" t="s">
@@ -1432,13 +1435,13 @@
         <v>87</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>34</v>
+        <v>12</v>
       </c>
       <c r="F25" s="3" t="s">
-        <v>34</v>
+        <v>137</v>
       </c>
       <c r="G25" s="3" t="s">
-        <v>35</v>
+        <v>13</v>
       </c>
       <c r="H25" s="3"/>
     </row>

</xml_diff>

<commit_message>
Date and time chnages
</commit_message>
<xml_diff>
--- a/terraform_modules_service_tracker V1.1.xlsx
+++ b/terraform_modules_service_tracker V1.1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ingrammicro-my.sharepoint.com/personal/jeetendra_wadhwani_ingrammicro_com/Documents/Desktop/terraform-aws-delivery/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="29" documentId="13_ncr:1_{F7EB1B05-2536-42C3-822D-4580F810F1EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{47E45865-DF43-4BC7-BCBE-D5981F8A2349}"/>
+  <xr:revisionPtr revIDLastSave="35" documentId="13_ncr:1_{F7EB1B05-2536-42C3-822D-4580F810F1EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E5BB8156-C9AF-40BD-B896-2C0B5F47F45E}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="268" uniqueCount="137">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="268" uniqueCount="138">
   <si>
     <t>Category</t>
   </si>
@@ -434,6 +434,9 @@
   </si>
   <si>
     <t>Check open SGs, public S3, unencrypted volumes</t>
+  </si>
+  <si>
+    <t>yes</t>
   </si>
 </sst>
 </file>
@@ -1057,10 +1060,10 @@
       <c r="H9" s="3"/>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A10" s="4" t="s">
+      <c r="A10" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="B10" s="5" t="s">
         <v>31</v>
       </c>
       <c r="C10" s="3" t="s">
@@ -1070,21 +1073,21 @@
         <v>33</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>34</v>
+        <v>12</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>34</v>
+        <v>12</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>35</v>
+        <v>13</v>
       </c>
       <c r="H10" s="3"/>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A11" s="4" t="s">
+      <c r="A11" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="B11" s="5" t="s">
         <v>36</v>
       </c>
       <c r="C11" s="3" t="s">
@@ -1094,13 +1097,13 @@
         <v>38</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>34</v>
+        <v>12</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>34</v>
+        <v>12</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>35</v>
+        <v>13</v>
       </c>
       <c r="H11" s="3"/>
     </row>
@@ -1419,10 +1422,10 @@
       <c r="H24" s="3"/>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A25" s="3" t="s">
+      <c r="A25" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="B25" s="3" t="s">
+      <c r="B25" s="5" t="s">
         <v>85</v>
       </c>
       <c r="C25" s="3" t="s">
@@ -1432,13 +1435,13 @@
         <v>87</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>34</v>
+        <v>12</v>
       </c>
       <c r="F25" s="3" t="s">
-        <v>34</v>
+        <v>137</v>
       </c>
       <c r="G25" s="3" t="s">
-        <v>35</v>
+        <v>13</v>
       </c>
       <c r="H25" s="3"/>
     </row>

</xml_diff>